<commit_message>
Correct council commendation to group honor; 40.5 point assessment
</commit_message>
<xml_diff>
--- a/入党积极分子考察测评/01-测评表/最新测评表_40.5分.xlsx
+++ b/入党积极分子考察测评/01-测评表/最新测评表_40.5分.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="R02f2c614dee54258"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="Rf6f0e175011a410e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1341,8 +1341,9 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="E20" s="23" t="str">
-        <x:v>同类取最高；同一活动媒体报道只计一次；不与前述获奖重复。
-2026.5校优秀共青团员2分；2025年4/5/6月五星文明寝室3次各1分；2025.12建材建工行业大会志愿者通报表扬2分。</x:v>
+        <x:v>同一类别取最高分;
+一次活动只计算一次媒体报道;
+不与前述获奖重复</x:v>
       </x:c>
       <x:c r="F20" s="3" t="n">
         <x:v>0</x:v>
@@ -1379,7 +1380,9 @@
       <x:c r="D22" s="4" t="s">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="E22" s="25"/>
+      <x:c r="E22" s="25" t="str">
+        <x:v>校优秀共青团员2分；2025年4、5、6月五星文明寝室集体荣誉各1分；建材建工大会志愿者集体通报表扬1分；台风送餐集体通报表扬1分。</x:v>
+      </x:c>
       <x:c r="F22" s="3" t="n">
         <x:v>7</x:v>
       </x:c>
@@ -1478,7 +1481,7 @@
       <x:c r="B28" s="59" t="str">
         <x:v>2024年9月确定为入党积极分子；2025年3月至今任研究生班级文体委员。研究10MW混合塔架结构与动力响应，获授权实用新型专利《一种风电塔筒加固结构》。
 在琼证明：学术活动11次、文体活动16次、思政活动7次。获2025年院级优秀歌手奖、2026年院级歌手二等奖、2025年校级师生合唱集体优胜奖、2026年院级拔河团体一等奖、校优秀共青团员；2025年4、5、6月三次五星文明寝室（院级集体荣誉）；另获研究生一、二等学业奖学金。
-普通志愿10次：2025.8.8科普（5h）、9.26招聘会（3.78h）、11.29歌手赛（7.88h）、12.12理事会（15h）、12.27田径运动会（4.6h）；2026.1.24—25插画艺术节（2天17.14h）、4.1和4.15飞盘赛（1.9h、8.6h）、4.26沙滩运动会（2.5h）。特殊志愿：2025.6.13台风送餐（4h）；理事会志愿获建材建工行业大会通报表扬（个人列名）。另有2025.12.21自行车赛志愿证书，记录0h。</x:v>
+普通志愿10次：2025.8.8科普（5h）、9.26招聘会（3.78h）、11.29歌手赛（7.88h）、12.12理事会（15h）、12.27田径运动会（4.6h）；2026.1.24—25插画艺术节（2天17.14h）、4.1和4.15飞盘赛（1.9h、8.6h）、4.26沙滩运动会（2.5h）。特殊志愿：2025.6.13台风送餐（4h），另获集体通报表扬；理事会志愿获建材建工行业大会集体通报表扬（名单含本人）。另有2025.12.21自行车赛志愿证书，记录0h。</x:v>
       </x:c>
       <x:c r="C28" s="59"/>
       <x:c r="D28" s="59"/>

</xml_diff>